<commit_message>
Fix epsilon number difference in SubtotalTests.PageBreaks/WithHeaders
The 9_plaindata.xlsx template contained two cells with a lot of decimal numbers
(H47 873.27000000000021 and I47 19627.879999999997), but gauges contained
rounded numbers (873.27 and 19627.88).

Therefore, the actual calculated value (from template) that had the number from
template (e.g. 873.27000000000021) while gauge contained 873.27. As a result, there
was a difference and SubtotalTests.PageBreaks plus few others failed.

This change updates the 9_plaindata.xlsx so it contains rounded numbers.

Same thing happened with the 91_plaindata.xlsx template, except test was
SubtotalTests.WithHeaders.
</commit_message>
<xml_diff>
--- a/tests/Templates/91_plaindata.xlsx
+++ b/tests/Templates/91_plaindata.xlsx
@@ -1737,10 +1737,10 @@
         <v>2121</v>
       </c>
       <c r="H47" s="19">
-        <v>873.27000000000021</v>
+        <v>873.27</v>
       </c>
       <c r="I47" s="19">
-        <v>19627.879999999997</v>
+        <v>19627.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>